<commit_message>
Ablation Study Experiments - Updated Results
</commit_message>
<xml_diff>
--- a/Ablation_results.xlsx
+++ b/Ablation_results.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\docs\Projects\DMP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\docs\Projects\PythonProject\DMP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDAC3B35-1B25-4F9B-854C-76F1052B1C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="REAL_Data" sheetId="4" r:id="rId1"/>
     <sheet name="PAPER_Data" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -71,7 +70,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -810,21 +809,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2573F877-A04D-4BA6-9D7F-8674A40D6360}">
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="1.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -850,7 +850,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -876,7 +876,7 @@
         <v>0.253</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>8</v>
       </c>
@@ -902,7 +902,7 @@
         <v>0.30099999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
@@ -928,7 +928,7 @@
         <v>0.28199999999999997</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
@@ -953,8 +953,26 @@
       <c r="H5" s="10">
         <v>0.23699999999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J5" s="36">
+        <v>0.9</v>
+      </c>
+      <c r="K5" s="38">
+        <v>0.68</v>
+      </c>
+      <c r="L5" s="37">
+        <v>0.78</v>
+      </c>
+      <c r="M5" s="36">
+        <v>0.87</v>
+      </c>
+      <c r="N5" s="38">
+        <v>0.41</v>
+      </c>
+      <c r="O5" s="37">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -979,8 +997,26 @@
       <c r="H6" s="4">
         <v>2.9000000000000001E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J6" s="28">
+        <v>0.78900000000000003</v>
+      </c>
+      <c r="K6" s="29">
+        <v>0.46899999999999997</v>
+      </c>
+      <c r="L6" s="30">
+        <v>0.58799999999999997</v>
+      </c>
+      <c r="M6" s="28">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="N6" s="29">
+        <v>0.02</v>
+      </c>
+      <c r="O6" s="30">
+        <v>2.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
@@ -1005,8 +1041,26 @@
       <c r="H7" s="12">
         <v>0.41799999999999998</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J7" s="31">
+        <v>0.72</v>
+      </c>
+      <c r="K7" s="32">
+        <v>0.56200000000000006</v>
+      </c>
+      <c r="L7" s="33">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="M7" s="31">
+        <v>0.46300000000000002</v>
+      </c>
+      <c r="N7" s="32">
+        <v>0.38</v>
+      </c>
+      <c r="O7" s="33">
+        <v>0.41799999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
@@ -1031,8 +1085,26 @@
       <c r="H8" s="7">
         <v>0.24199999999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J8" s="31">
+        <v>0.75</v>
+      </c>
+      <c r="K8" s="32">
+        <v>0.65600000000000003</v>
+      </c>
+      <c r="L8" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="M8" s="31">
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="N8" s="32">
+        <v>0.22</v>
+      </c>
+      <c r="O8" s="33">
+        <v>0.24199999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="8" t="s">
         <v>13</v>
       </c>
@@ -1057,8 +1129,26 @@
       <c r="H9" s="10">
         <v>0.189</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J9" s="36">
+        <v>0.96</v>
+      </c>
+      <c r="K9" s="38">
+        <v>0.84</v>
+      </c>
+      <c r="L9" s="37">
+        <v>0.9</v>
+      </c>
+      <c r="M9" s="36">
+        <v>1</v>
+      </c>
+      <c r="N9" s="38">
+        <v>0.7</v>
+      </c>
+      <c r="O9" s="37">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>14</v>
       </c>
@@ -1083,8 +1173,26 @@
       <c r="H10" s="4">
         <v>0.22500000000000001</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J10" s="28">
+        <v>0.90500000000000003</v>
+      </c>
+      <c r="K10" s="29">
+        <v>0.51400000000000001</v>
+      </c>
+      <c r="L10" s="30">
+        <v>0.65500000000000003</v>
+      </c>
+      <c r="M10" s="28">
+        <v>0.29399999999999998</v>
+      </c>
+      <c r="N10" s="29">
+        <v>0.182</v>
+      </c>
+      <c r="O10" s="30">
+        <v>0.22500000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
@@ -1109,8 +1217,26 @@
       <c r="H11" s="7">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J11" s="31">
+        <v>0.88200000000000001</v>
+      </c>
+      <c r="K11" s="35">
+        <v>0.81100000000000005</v>
+      </c>
+      <c r="L11" s="33">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="M11" s="31">
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="N11" s="32">
+        <v>0.34499999999999997</v>
+      </c>
+      <c r="O11" s="33">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
@@ -1135,8 +1261,26 @@
       <c r="H12" s="12">
         <v>0.47399999999999998</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J12" s="31">
+        <v>0.88200000000000001</v>
+      </c>
+      <c r="K12" s="35">
+        <v>0.81100000000000005</v>
+      </c>
+      <c r="L12" s="33">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="M12" s="31">
+        <v>0.54800000000000004</v>
+      </c>
+      <c r="N12" s="32">
+        <v>0.41799999999999998</v>
+      </c>
+      <c r="O12" s="33">
+        <v>0.47399999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="8" t="s">
         <v>14</v>
       </c>
@@ -1160,6 +1304,24 @@
       </c>
       <c r="H13" s="10">
         <v>0.36599999999999999</v>
+      </c>
+      <c r="J13" s="36">
+        <v>0.91</v>
+      </c>
+      <c r="K13" s="34">
+        <v>0.81</v>
+      </c>
+      <c r="L13" s="37">
+        <v>0.86</v>
+      </c>
+      <c r="M13" s="36">
+        <v>0.87</v>
+      </c>
+      <c r="N13" s="38">
+        <v>0.62</v>
+      </c>
+      <c r="O13" s="37">
+        <v>0.72</v>
       </c>
     </row>
   </sheetData>
@@ -1168,21 +1330,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1208,7 +1370,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="22" t="s">
         <v>8</v>
       </c>
@@ -1234,7 +1396,7 @@
         <v>0.253</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="23" t="s">
         <v>8</v>
       </c>
@@ -1260,7 +1422,7 @@
         <v>0.30099999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="23" t="s">
         <v>8</v>
       </c>
@@ -1286,7 +1448,7 @@
         <v>0.28199999999999997</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="24" t="s">
         <v>8</v>
       </c>
@@ -1312,7 +1474,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="22" t="s">
         <v>13</v>
       </c>
@@ -1338,7 +1500,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="23" t="s">
         <v>13</v>
       </c>
@@ -1364,7 +1526,7 @@
         <v>0.41799999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="23" t="s">
         <v>13</v>
       </c>
@@ -1390,7 +1552,7 @@
         <v>0.24199999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="24" t="s">
         <v>13</v>
       </c>
@@ -1416,7 +1578,7 @@
         <v>0.82</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="22" t="s">
         <v>14</v>
       </c>
@@ -1442,7 +1604,7 @@
         <v>0.22500000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="23" t="s">
         <v>14</v>
       </c>
@@ -1468,7 +1630,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="23" t="s">
         <v>14</v>
       </c>
@@ -1494,7 +1656,7 @@
         <v>0.47399999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="24" t="s">
         <v>14</v>
       </c>

</xml_diff>